<commit_message>
Stok menipis dan routing
</commit_message>
<xml_diff>
--- a/dataset_vape_shop_200_produk.xlsx
+++ b/dataset_vape_shop_200_produk.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Ridho\svp-stock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB501D29-E9AE-46A5-A16C-8DBE8384CAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B3C7624-A919-4E94-8AE7-18F13FAF02DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Produk Vape" sheetId="1" r:id="rId1"/>

</xml_diff>